<commit_message>
expand run manifest generator
</commit_message>
<xml_diff>
--- a/hf_manifest.xlsx
+++ b/hf_manifest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://curtin-my.sharepoint.com/personal/21550803_student_curtin_edu_au/Documents/Documents/University/MLaaS/MLaaS-Dataset-Generator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_7041301BD57BFA0B679A2211595ED87656DEF6B7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BB2A805B-2160-4155-A543-6C24DDA3BFF1}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_7041301BD57BFA0B679A2211595ED87656DEF6B7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D4ED306-10C2-442A-9855-BA1D38BE994F}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5627,6 +5627,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5917,6 +5921,8 @@
   <dimension ref="A1:AL701"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="4" max="4" width="99.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="52.140625" bestFit="1" customWidth="1"/>
     <col min="34" max="34" width="78.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>